<commit_message>
- adds support for Orbiter smart roaster - adds popup on missing bean information on START if plus is connected
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$133</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$134</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="410">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -689,6 +689,12 @@
   </si>
   <si>
     <t xml:space="preserve">sends &lt;value&gt; to &lt;target&gt; via the Kaleido Serial or Network protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orbiter(&lt;cmd&gt;[,&lt;value&gt;[,&lt;param&gt;]])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sends &lt;cmd&gt; (1byte in HEX) and optional &lt;value&gt; (0-65535) and &lt;param&gt; (0-255) to Orbiter</t>
   </si>
   <si>
     <t xml:space="preserve">shellyrelay(n,b)</t>
@@ -2167,7 +2173,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C168"/>
+  <dimension ref="A1:C169"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -2635,7 +2641,7 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="1" t="s">
+      <c r="B59" s="3" t="s">
         <v>213</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -2654,29 +2660,29 @@
       <c r="A61" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="C61" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="C62" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B63" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="C63" s="1" t="s">
         <v>224</v>
       </c>
     </row>
@@ -2687,11 +2693,11 @@
       <c r="B64" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C64" s="1" t="s">
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="3" t="s">
         <v>228</v>
       </c>
@@ -2772,17 +2778,17 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1" t="s">
+      <c r="B75" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="C75" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="C75" s="1" t="s">
+    </row>
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="3" t="s">
         <v>251</v>
       </c>
@@ -2808,69 +2814,69 @@
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C80" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="B80" s="3" t="s">
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B81" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C80" s="1" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="3" t="s">
-        <v>129</v>
-      </c>
       <c r="C81" s="1" t="s">
-        <v>130</v>
+        <v>260</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3" t="s">
-        <v>259</v>
+        <v>137</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>260</v>
+        <v>138</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2922,16 +2928,16 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1" t="s">
+      <c r="B93" s="3" t="s">
         <v>273</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>214</v>
+        <v>274</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>216</v>
@@ -2939,40 +2945,40 @@
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>276</v>
+        <v>218</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="C96" s="1" t="s">
         <v>278</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B97" s="3" t="s">
+      <c r="C97" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B98" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C97" s="1" t="s">
+      <c r="C98" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B98" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,18 +3007,18 @@
     </row>
     <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="3" t="s">
-        <v>131</v>
+        <v>289</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>132</v>
+        <v>290</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="3" t="s">
-        <v>289</v>
+        <v>131</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>290</v>
+        <v>132</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3177,15 +3183,15 @@
     </row>
     <row r="124" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="3" t="s">
-        <v>133</v>
+        <v>331</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="3" t="s">
-        <v>332</v>
+        <v>133</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>333</v>
@@ -3193,18 +3199,18 @@
     </row>
     <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3" t="s">
-        <v>137</v>
+        <v>334</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>138</v>
+        <v>335</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3" t="s">
-        <v>334</v>
+        <v>137</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>335</v>
+        <v>138</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3360,17 +3366,17 @@
       </c>
     </row>
     <row r="147" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="1" t="s">
+      <c r="B147" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="B147" s="3" t="s">
+      <c r="C147" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="C147" s="1" t="s">
+    </row>
+    <row r="148" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="1" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="148" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="3" t="s">
         <v>377</v>
       </c>
@@ -3428,15 +3434,15 @@
     </row>
     <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="3" t="s">
-        <v>240</v>
+        <v>391</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="3" t="s">
-        <v>392</v>
+        <v>242</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>393</v>
@@ -3452,26 +3458,26 @@
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
-        <v>249</v>
+        <v>396</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="1" t="s">
-        <v>397</v>
-      </c>
       <c r="B159" s="3" t="s">
-        <v>389</v>
+        <v>251</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="1" t="s">
+        <v>399</v>
+      </c>
       <c r="B160" s="3" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>400</v>
@@ -3479,69 +3485,77 @@
     </row>
     <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="3" t="s">
-        <v>379</v>
+        <v>401</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="1" t="s">
-        <v>402</v>
-      </c>
       <c r="B162" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="B163" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C162" s="1" t="s">
+      <c r="C163" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B163" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="C163" s="1" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="3" t="s">
-        <v>131</v>
+        <v>405</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>132</v>
+        <v>406</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>405</v>
+        <v>134</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>138</v>
+        <v>407</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>406</v>
+        <v>137</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>407</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B169" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- adds MQTT support - adds support for ROEST sample and production roasters
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$134</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$135</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="412">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -701,6 +701,12 @@
   </si>
   <si>
     <t xml:space="preserve">switches Shelly plug number &lt;n&gt; ON if b is true or 1, and OFF otherwise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">publish(&lt;topic&gt;, &lt;value&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">converts the given data to JSON and publish it on the MQTT server to the given topic</t>
   </si>
   <si>
     <t xml:space="preserve">Hottop Heater</t>
@@ -2173,7 +2179,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C169"/>
+  <dimension ref="A1:C170"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -2649,7 +2655,7 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="1" t="s">
+      <c r="B60" s="3" t="s">
         <v>215</v>
       </c>
       <c r="C60" s="1" t="s">
@@ -2668,29 +2674,29 @@
       <c r="A62" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="C62" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="C63" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B64" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="C64" s="1" t="s">
         <v>226</v>
       </c>
     </row>
@@ -2701,11 +2707,11 @@
       <c r="B65" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="C65" s="1" t="s">
+    </row>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="3" t="s">
         <v>230</v>
       </c>
@@ -2786,17 +2792,17 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="s">
+      <c r="B76" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="C76" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="C76" s="1" t="s">
+    </row>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="3" t="s">
         <v>253</v>
       </c>
@@ -2822,69 +2828,69 @@
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C81" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="B81" s="3" t="s">
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B82" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C81" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B82" s="3" t="s">
-        <v>129</v>
-      </c>
       <c r="C82" s="1" t="s">
-        <v>130</v>
+        <v>262</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="3" t="s">
-        <v>261</v>
+        <v>137</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>262</v>
+        <v>138</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2936,16 +2942,16 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1" t="s">
+      <c r="B94" s="3" t="s">
         <v>275</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>216</v>
+        <v>276</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>218</v>
@@ -2953,40 +2959,40 @@
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>278</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B97" s="3" t="s">
+      <c r="C97" s="1" t="s">
         <v>280</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B98" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B98" s="3" t="s">
+      <c r="C98" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B99" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C98" s="1" t="s">
+      <c r="C99" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B99" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,18 +3021,18 @@
     </row>
     <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="3" t="s">
-        <v>131</v>
+        <v>291</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>132</v>
+        <v>292</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="3" t="s">
-        <v>291</v>
+        <v>131</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>292</v>
+        <v>132</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3191,15 +3197,15 @@
     </row>
     <row r="125" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="3" t="s">
-        <v>133</v>
+        <v>333</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3" t="s">
-        <v>334</v>
+        <v>133</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>335</v>
@@ -3207,18 +3213,18 @@
     </row>
     <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3" t="s">
-        <v>137</v>
+        <v>336</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>138</v>
+        <v>337</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="3" t="s">
-        <v>336</v>
+        <v>137</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>337</v>
+        <v>138</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3374,17 +3380,17 @@
       </c>
     </row>
     <row r="148" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="1" t="s">
+      <c r="B148" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="B148" s="3" t="s">
+      <c r="C148" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="C148" s="1" t="s">
+    </row>
+    <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="1" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="3" t="s">
         <v>379</v>
       </c>
@@ -3442,15 +3448,15 @@
     </row>
     <row r="156" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="3" t="s">
-        <v>242</v>
+        <v>393</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="3" t="s">
-        <v>394</v>
+        <v>244</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>395</v>
@@ -3466,26 +3472,26 @@
     </row>
     <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="3" t="s">
-        <v>251</v>
+        <v>398</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="1" t="s">
-        <v>399</v>
-      </c>
       <c r="B160" s="3" t="s">
-        <v>391</v>
+        <v>253</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="1" t="s">
+        <v>401</v>
+      </c>
       <c r="B161" s="3" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>402</v>
@@ -3493,69 +3499,77 @@
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="3" t="s">
-        <v>381</v>
+        <v>403</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="1" t="s">
-        <v>404</v>
-      </c>
       <c r="B163" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B164" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C163" s="1" t="s">
+      <c r="C164" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B164" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="C164" s="1" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3" t="s">
-        <v>131</v>
+        <v>407</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>132</v>
+        <v>408</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>407</v>
+        <v>134</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>138</v>
+        <v>409</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>408</v>
+        <v>137</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>409</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B170" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- adds RoastHubs support - tightens license from GPLv3 to AGPLv3
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="414">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -1330,6 +1330,12 @@
   </si>
   <si>
     <t xml:space="preserve">shows/hides the events of the background profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload2RoastHubs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upload current loaded profile to RoastHubs</t>
   </si>
   <si>
     <t xml:space="preserve">RC Command</t>
@@ -2179,7 +2185,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C170"/>
+  <dimension ref="A1:C171"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -3388,17 +3394,17 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="1" t="s">
+      <c r="B149" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="B149" s="3" t="s">
+      <c r="C149" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="C149" s="1" t="s">
+    </row>
+    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="1" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="3" t="s">
         <v>381</v>
       </c>
@@ -3456,15 +3462,15 @@
     </row>
     <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="3" t="s">
-        <v>244</v>
+        <v>395</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
-        <v>396</v>
+        <v>244</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>397</v>
@@ -3480,26 +3486,26 @@
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B161" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="C160" s="1" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="B161" s="3" t="s">
-        <v>393</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="B162" s="3" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>404</v>
@@ -3507,69 +3513,77 @@
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3" t="s">
-        <v>383</v>
+        <v>405</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="1" t="s">
-        <v>406</v>
-      </c>
       <c r="B164" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B165" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C164" s="1" t="s">
+      <c r="C165" s="1" t="s">
         <v>130</v>
-      </c>
-    </row>
-    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B165" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>131</v>
+        <v>409</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>132</v>
+        <v>410</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B167" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>409</v>
+        <v>134</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>138</v>
+        <v>411</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="3" t="s">
-        <v>410</v>
+        <v>137</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>411</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B171" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>413</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- adds Artisan Commands pidDerivativeFilter, pidDerivativeLimit, pidILF, pidIWP, and pidIRoC - fixes some links - fixes small keyboard mode issue - more renaming
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Commands" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$135</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">Commands!$C$140</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="424">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -997,6 +997,36 @@
   </si>
   <si>
     <t xml:space="preserve">sets the beta and gamma parameters of the PID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidDerivativeFilter(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets derivative filter size;  0 &lt;= n &lt; 6 (n:int)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidDerivativeLimit(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets derivative limit (Dlimit); n &gt;= 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidILF(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets integral limit factor; 0&lt;=n&lt;=1 (n:float)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidIWP(&lt;bool&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggles integral windup prevention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pidIRoC(&lt;bool&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toggles integral reset on target</t>
   </si>
   <si>
     <t xml:space="preserve">adjustSV(&lt;float&gt;)</t>
@@ -2185,7 +2215,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C171"/>
+  <dimension ref="A1:C176"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -3211,66 +3241,66 @@
     </row>
     <row r="126" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3" t="s">
-        <v>133</v>
+        <v>335</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="3" t="s">
-        <v>137</v>
+        <v>339</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>138</v>
+        <v>340</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="3" t="s">
-        <v>342</v>
+        <v>133</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="3" t="s">
-        <v>346</v>
+        <v>137</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>347</v>
+        <v>138</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,49 +3432,49 @@
       </c>
     </row>
     <row r="150" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="1" t="s">
+      <c r="B150" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="B150" s="3" t="s">
+      <c r="C150" s="1" t="s">
         <v>381</v>
-      </c>
-      <c r="C150" s="1" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C151" s="1" t="s">
         <v>383</v>
-      </c>
-      <c r="C151" s="1" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="C152" s="1" t="s">
         <v>385</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>387</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B154" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="C154" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="C154" s="1" t="s">
+    </row>
+    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="1" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="3" t="s">
         <v>391</v>
       </c>
@@ -3470,120 +3500,160 @@
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
-        <v>244</v>
+        <v>397</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="3" t="s">
-        <v>253</v>
+        <v>403</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="1" t="s">
-        <v>403</v>
-      </c>
       <c r="B162" s="3" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3" t="s">
-        <v>405</v>
+        <v>244</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B164" s="3" t="s">
-        <v>385</v>
+        <v>408</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="1" t="s">
-        <v>408</v>
-      </c>
       <c r="B165" s="3" t="s">
-        <v>129</v>
+        <v>410</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>130</v>
+        <v>411</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>409</v>
+        <v>253</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="s">
+        <v>413</v>
+      </c>
       <c r="B167" s="3" t="s">
-        <v>131</v>
+        <v>405</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>132</v>
+        <v>414</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>133</v>
+        <v>415</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>134</v>
+        <v>416</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>135</v>
+        <v>395</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="s">
+        <v>418</v>
+      </c>
       <c r="B170" s="3" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="3" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>413</v>
+        <v>420</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B172" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C172" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B173" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B174" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C174" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B175" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B176" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- switch acaia COSMO to streaming mode - RoastHubs profile upload respecting current curve smoothing settings - fixed size login dialogs - adds Artisan Commands `zoom(<x>[,<y>])`, `pan(<x>[,<y>])`, `center(<x>,<y>[,<clamp>])`, `clamp(<n>)`, `followMode(<bool>)`, and `followModePanning(<x>[,<y>])` to update the canvas perspective - adds Artisan Commands `home`, `back` and `forward` to operate the navigation bar - improved PID buttons layout - updated icons and translations - lib updates
</commit_message>
<xml_diff>
--- a/doc/help_dialogs/Input_files/eventbuttons.xlsx
+++ b/doc/help_dialogs/Input_files/eventbuttons.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="442">
   <si>
     <t xml:space="preserve">EVENT CUSTOM BUTTONS</t>
   </si>
@@ -1366,6 +1366,60 @@
   </si>
   <si>
     <t xml:space="preserve">upload current loaded profile to RoastHubs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zoom(&lt;x&gt;[,&lt;y&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zooms the canvas by factor &lt;x&gt; horizontally and the optional &lt;y&gt; vertically. &lt;y&gt; defaults to &lt;x&gt;.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pan(&lt;x&gt;[,&lt;y&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pans the canvas by factor &lt;x&gt; horizontally and the optional &lt;y&gt; vertically. A factor 0 does not apply any panning, a factor 1 moves by one full screen to the left/bottom, a factor -1 by one full screen to the right/top. &lt;y&gt; defaults to &lt;x&gt;.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">center(&lt;x&gt;,&lt;y&gt;[,&lt;clamp&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">centers canvas and then applies panning according to the given x/y parameters in horizontal and vertical direction. 0: no panning, 1: pan canvas one full screen to the left/bottom, -1: pan canvas one full screen to the right/top. If &lt;clamp&gt; is 0 the canvas is centered w.r.t. both axis limits. If not recording, and &lt;clamp&gt; i -1 the canvas is centered only horizontally wr.t. its x-axis limits and with clamp in {1,..,4} w.r.t. to both axis limits. While recording if &lt;clamp&gt; is -1 the canvas is centered horizontally to the current time, if 1 also centered to current BT, 2 current ET, 3 current BT RoR, 4 current ET RoR. &lt;clamp&gt; defaults to -1 if xy-cursor widget is clamped to any temp or RoR curve (z-key), 0 if zoom follow is OFF and xy-cursor not clamped, 1-4 if zoom follow is ON and xy-cursor not clamped, centering on the value zoom followed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clamp(&lt;n&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">set xy cursor clamp mode (shortcut key z) to 0: off, 1: BT@x, 2: ET@x, 3: BTB@x, 4: ETB@x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">followMode(&lt;bool&gt;)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enables/disables follow mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">followModePanning(&lt;x&gt;[,&lt;y&gt;])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sets additional panning in horizontal and vertical direction, applied in follow mode after the centering. 0: no panning, 1: pan canvas one full screen to the left/bottom, -1: pan canvas one full screen to the right/top. &lt;y&gt; defaults to &lt;x&gt;.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toolbar home action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toolbar back action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toolbar forward action</t>
   </si>
   <si>
     <t xml:space="preserve">RC Command</t>
@@ -2215,7 +2269,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C176"/>
+  <dimension ref="A1:C185"/>
   <sheetFormatPr defaultColWidth="9.2734375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.73"/>
@@ -3472,191 +3526,266 @@
       </c>
     </row>
     <row r="155" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="1" t="s">
+      <c r="B155" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="B155" s="3" t="s">
+      <c r="C155" s="1" t="s">
         <v>391</v>
-      </c>
-      <c r="C155" s="1" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B156" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C156" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="C156" s="1" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C157" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="C157" s="1" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C158" s="1" t="s">
         <v>397</v>
-      </c>
-      <c r="C158" s="1" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="C159" s="1" t="s">
         <v>399</v>
-      </c>
-      <c r="C159" s="1" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C160" s="1" t="s">
         <v>401</v>
-      </c>
-      <c r="C160" s="1" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="C161" s="1" t="s">
         <v>403</v>
-      </c>
-      <c r="C161" s="1" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="C162" s="1" t="s">
         <v>405</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="3" t="s">
-        <v>244</v>
+        <v>406</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1" t="s">
+        <v>408</v>
+      </c>
       <c r="B164" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="3" t="s">
-        <v>253</v>
+        <v>413</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="1" t="s">
-        <v>413</v>
-      </c>
       <c r="B167" s="3" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B168" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="3" t="s">
-        <v>395</v>
+        <v>419</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="1" t="s">
-        <v>418</v>
-      </c>
       <c r="B170" s="3" t="s">
-        <v>129</v>
+        <v>421</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>130</v>
+        <v>422</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="3" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B172" s="3" t="s">
-        <v>131</v>
+        <v>244</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>132</v>
+        <v>425</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B173" s="3" t="s">
-        <v>133</v>
+        <v>426</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>134</v>
+        <v>427</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B174" s="3" t="s">
-        <v>135</v>
+        <v>428</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B175" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B177" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="C177" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B178" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="C178" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B179" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C179" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B180" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="C180" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="181" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B181" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C181" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="182" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B182" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C182" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="183" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B183" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C183" s="1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="184" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B184" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C175" s="1" t="s">
+      <c r="C184" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B176" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="C176" s="1" t="s">
-        <v>423</v>
+    <row r="185" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B185" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>441</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C158" r:id="rId1" display="ETB@x"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>